<commit_message>
Overhaul rate sheet keys to short names, simplify rate lookup, combine REDC/REDE to RED
</commit_message>
<xml_diff>
--- a/Plans/CompRefTable.xlsx
+++ b/Plans/CompRefTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Conversion\summit-takeoff-poc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve\source\repos\PrinceCorwin\VANTAGE\Plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4A326D-52AA-4C20-BECA-D9D6FB143C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE67D24D-9E82-4886-AF58-8DB955E05EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52736E01-4DB2-4534-8411-C88F195D644A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{52736E01-4DB2-4534-8411-C88F195D644A}"/>
   </bookViews>
   <sheets>
     <sheet name="CompRef" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="445">
   <si>
     <t>ConnType</t>
   </si>
@@ -1018,12 +1018,6 @@
     <t>NIPPLE SCH 10S 316/316L SS PBE 3 LONG</t>
   </si>
   <si>
-    <t>REDC</t>
-  </si>
-  <si>
-    <t>REDE</t>
-  </si>
-  <si>
     <t>SAFSHW</t>
   </si>
   <si>
@@ -1291,12 +1285,6 @@
     <t>FO, FLOW ORIFICE, RESTRICTION ORIFICE, ORIFICE PLATE, FLOW RESTRICTION, RESTR ORIFICE, REST ORIFICE, RO, FLOW ORIFICE NON-HYG, RESTRICTION NON-HYG, FLOW ELEMENT, FE ORIFICE, ORIFICE ELEMENT</t>
   </si>
   <si>
-    <t>CONC REDUCER, CONCENTRIC REDUCER, CONC RED, CON RED, REDUCER CONC, RED CONC, CONCENTRIC RED, CONC REDCR, CON REDCR, REDCR CONC</t>
-  </si>
-  <si>
-    <t>ECC REDUCER, ECCENTRIC REDUCER, ECC RED, REDUCER ECC, RED ECC, ECCENTRIC RED, ECC REDCR, REDCR ECC, ECCENTRIC REDCR</t>
-  </si>
-  <si>
     <t>REGULATOR VALVE, REG VALVE, REG VLV, PRESSURE REGULATOR, PRESS REG, PRV NON-HYG, REGULATOR NON-HYG, PRESSURE REG VLV, PIRV, PRESSURE IND REG VALVE, PRESS IND REG VLV</t>
   </si>
   <si>
@@ -1388,6 +1376,12 @@
   </si>
   <si>
     <t>SPT</t>
+  </si>
+  <si>
+    <t>RED</t>
+  </si>
+  <si>
+    <t>CONC REDUCER, CONCENTRIC REDUCER, CONC RED, CON RED, REDUCER CONC, RED CONC, CONCENTRIC RED, CONC REDCR, CON REDCR, REDCR CONC, ECC REDUCER, ECCENTRIC REDUCER, ECC RED, REDUCER ECC, RED ECC, ECCENTRIC RED, ECC REDCR, REDCR ECC, ECCENTRIC REDCR</t>
   </si>
 </sst>
 </file>
@@ -1591,9 +1585,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{291D72AD-DD03-44B3-B302-066A40CDCB63}" name="Table2_12" displayName="Table2_12" ref="A1:E303" tableType="queryTable" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:E303" xr:uid="{291D72AD-DD03-44B3-B302-066A40CDCB63}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E303">
-    <sortCondition ref="B1:B303"/>
-  </sortState>
   <tableColumns count="5">
     <tableColumn id="17" xr3:uid="{54521D18-D32C-4F40-BF10-1558C1E0C78E}" uniqueName="17" name="Description" queryTableFieldId="17" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{25857F6B-ED8A-49F5-989F-BD07682CA5EA}" uniqueName="3" name="Component" queryTableFieldId="27" dataDxfId="7"/>
@@ -1923,33 +1914,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5DB19FA-DF86-4DC5-B9D6-4C6A64D26755}">
   <dimension ref="A1:E303"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="78.28515625" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="83.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="78.26171875" customWidth="1"/>
+    <col min="2" max="2" width="15.26171875" customWidth="1"/>
+    <col min="3" max="3" width="15.26171875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.41796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="83.83984375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B1" t="s">
         <v>255</v>
       </c>
       <c r="C1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1963,10 +1954,10 @@
         <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1980,10 +1971,10 @@
         <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1997,10 +1988,10 @@
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2014,10 +2005,10 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -2031,10 +2022,10 @@
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2048,10 +2039,10 @@
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -2065,10 +2056,10 @@
         <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -2082,10 +2073,10 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -2099,10 +2090,10 @@
         <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>289</v>
       </c>
@@ -2116,10 +2107,10 @@
         <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -2133,10 +2124,10 @@
         <v>15</v>
       </c>
       <c r="E12" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -2150,10 +2141,10 @@
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -2167,10 +2158,10 @@
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -2184,10 +2175,10 @@
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -2201,10 +2192,10 @@
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -2218,10 +2209,10 @@
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -2235,10 +2226,10 @@
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -2252,10 +2243,10 @@
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -2269,10 +2260,10 @@
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -2286,10 +2277,10 @@
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -2303,10 +2294,10 @@
         <v>18</v>
       </c>
       <c r="E22" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2320,10 +2311,10 @@
         <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -2337,10 +2328,10 @@
         <v>8</v>
       </c>
       <c r="E24" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -2354,10 +2345,10 @@
         <v>8</v>
       </c>
       <c r="E25" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -2371,10 +2362,10 @@
         <v>3</v>
       </c>
       <c r="E26" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -2388,15 +2379,15 @@
         <v>3</v>
       </c>
       <c r="E27" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="B28" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -2405,15 +2396,15 @@
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="B29" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C29">
         <v>2</v>
@@ -2422,15 +2413,15 @@
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="B30" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C30">
         <v>2</v>
@@ -2439,15 +2430,15 @@
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="B31" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C31">
         <v>2</v>
@@ -2456,15 +2447,15 @@
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="B32" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C32">
         <v>2</v>
@@ -2473,15 +2464,15 @@
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="B33" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C33">
         <v>2</v>
@@ -2490,15 +2481,15 @@
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
+        <v>427</v>
+      </c>
+      <c r="B34" t="s">
         <v>431</v>
-      </c>
-      <c r="B34" t="s">
-        <v>435</v>
       </c>
       <c r="C34">
         <v>2</v>
@@ -2507,15 +2498,15 @@
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="B35" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C35">
         <v>2</v>
@@ -2524,15 +2515,15 @@
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="B36" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -2541,15 +2532,15 @@
         <v>8</v>
       </c>
       <c r="E36" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B37" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C37">
         <v>2</v>
@@ -2558,15 +2549,15 @@
         <v>8</v>
       </c>
       <c r="E37" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="B38" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="C38">
         <v>2</v>
@@ -2575,15 +2566,15 @@
         <v>8</v>
       </c>
       <c r="E38" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>268</v>
       </c>
       <c r="B39" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -2592,7 +2583,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -2609,7 +2600,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
         <v>184</v>
       </c>
@@ -2623,7 +2614,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
         <v>178</v>
       </c>
@@ -2637,7 +2628,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
         <v>179</v>
       </c>
@@ -2651,7 +2642,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
         <v>180</v>
       </c>
@@ -2665,7 +2656,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
         <v>181</v>
       </c>
@@ -2679,7 +2670,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" t="s">
         <v>261</v>
       </c>
@@ -2693,7 +2684,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" t="s">
         <v>185</v>
       </c>
@@ -2707,7 +2698,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" t="s">
         <v>186</v>
       </c>
@@ -2721,7 +2712,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
         <v>187</v>
       </c>
@@ -2735,7 +2726,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
         <v>290</v>
       </c>
@@ -2749,7 +2740,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
         <v>188</v>
       </c>
@@ -2763,7 +2754,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
         <v>189</v>
       </c>
@@ -2777,7 +2768,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
         <v>175</v>
       </c>
@@ -2794,7 +2785,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" t="s">
         <v>176</v>
       </c>
@@ -2811,7 +2802,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" t="s">
         <v>182</v>
       </c>
@@ -2828,7 +2819,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" t="s">
         <v>190</v>
       </c>
@@ -2842,12 +2833,12 @@
         <v>233</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" t="s">
         <v>304</v>
       </c>
       <c r="B57" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C57">
         <v>2</v>
@@ -2859,12 +2850,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" t="s">
         <v>7</v>
       </c>
       <c r="B58" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C58">
         <v>2</v>
@@ -2876,12 +2867,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" t="s">
         <v>9</v>
       </c>
       <c r="B59" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C59">
         <v>2</v>
@@ -2893,12 +2884,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" t="s">
         <v>38</v>
       </c>
       <c r="B60" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C60">
         <v>2</v>
@@ -2910,12 +2901,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" t="s">
         <v>39</v>
       </c>
       <c r="B61" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C61">
         <v>2</v>
@@ -2927,12 +2918,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" t="s">
         <v>40</v>
       </c>
       <c r="B62" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C62">
         <v>2</v>
@@ -2944,12 +2935,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" t="s">
         <v>4</v>
       </c>
       <c r="B63" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C63">
         <v>2</v>
@@ -2961,12 +2952,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" t="s">
         <v>5</v>
       </c>
       <c r="B64" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C64">
         <v>2</v>
@@ -2978,12 +2969,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" t="s">
         <v>6</v>
       </c>
       <c r="B65" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C65">
         <v>2</v>
@@ -2995,7 +2986,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" t="s">
         <v>191</v>
       </c>
@@ -3009,12 +3000,12 @@
         <v>284</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="B67" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="C67">
         <v>2</v>
@@ -3023,15 +3014,15 @@
         <v>86</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="B68" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="C68">
         <v>2</v>
@@ -3040,15 +3031,15 @@
         <v>80</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="B69" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="C69">
         <v>2</v>
@@ -3057,10 +3048,10 @@
         <v>99</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" t="s">
         <v>293</v>
       </c>
@@ -3071,10 +3062,10 @@
         <v>0</v>
       </c>
       <c r="E70" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" t="s">
         <v>45</v>
       </c>
@@ -3088,10 +3079,10 @@
         <v>46</v>
       </c>
       <c r="E71" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" t="s">
         <v>48</v>
       </c>
@@ -3105,10 +3096,10 @@
         <v>50</v>
       </c>
       <c r="E72" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" t="s">
         <v>49</v>
       </c>
@@ -3122,10 +3113,10 @@
         <v>50</v>
       </c>
       <c r="E73" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" t="s">
         <v>43</v>
       </c>
@@ -3139,10 +3130,10 @@
         <v>44</v>
       </c>
       <c r="E74" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" t="s">
         <v>51</v>
       </c>
@@ -3156,10 +3147,10 @@
         <v>44</v>
       </c>
       <c r="E75" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" t="s">
         <v>52</v>
       </c>
@@ -3173,10 +3164,10 @@
         <v>44</v>
       </c>
       <c r="E76" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" t="s">
         <v>53</v>
       </c>
@@ -3190,10 +3181,10 @@
         <v>44</v>
       </c>
       <c r="E77" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" t="s">
         <v>54</v>
       </c>
@@ -3207,10 +3198,10 @@
         <v>44</v>
       </c>
       <c r="E78" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" t="s">
         <v>300</v>
       </c>
@@ -3221,13 +3212,13 @@
         <v>2</v>
       </c>
       <c r="D79" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E79" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A80" t="s">
         <v>301</v>
       </c>
@@ -3238,15 +3229,15 @@
         <v>2</v>
       </c>
       <c r="D80" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E80" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B81" t="s">
         <v>305</v>
@@ -3258,10 +3249,10 @@
         <v>44</v>
       </c>
       <c r="E81" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" t="s">
         <v>306</v>
       </c>
@@ -3272,15 +3263,15 @@
         <v>2</v>
       </c>
       <c r="D82" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E82" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A83" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B83" t="s">
         <v>305</v>
@@ -3292,10 +3283,10 @@
         <v>50</v>
       </c>
       <c r="E83" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A84" t="s">
         <v>294</v>
       </c>
@@ -3309,10 +3300,10 @@
         <v>15</v>
       </c>
       <c r="E84" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A85" t="s">
         <v>295</v>
       </c>
@@ -3326,10 +3317,10 @@
         <v>15</v>
       </c>
       <c r="E85" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A86" t="s">
         <v>296</v>
       </c>
@@ -3343,10 +3334,10 @@
         <v>15</v>
       </c>
       <c r="E86" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A87" t="s">
         <v>257</v>
       </c>
@@ -3360,10 +3351,10 @@
         <v>15</v>
       </c>
       <c r="E87" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A88" t="s">
         <v>258</v>
       </c>
@@ -3377,10 +3368,10 @@
         <v>15</v>
       </c>
       <c r="E88" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" t="s">
         <v>297</v>
       </c>
@@ -3394,10 +3385,10 @@
         <v>15</v>
       </c>
       <c r="E89" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" t="s">
         <v>259</v>
       </c>
@@ -3411,10 +3402,10 @@
         <v>15</v>
       </c>
       <c r="E90" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A91" t="s">
         <v>41</v>
       </c>
@@ -3428,10 +3419,10 @@
         <v>15</v>
       </c>
       <c r="E91" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A92" t="s">
         <v>74</v>
       </c>
@@ -3445,10 +3436,10 @@
         <v>15</v>
       </c>
       <c r="E92" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A93" t="s">
         <v>75</v>
       </c>
@@ -3462,10 +3453,10 @@
         <v>15</v>
       </c>
       <c r="E93" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A94" t="s">
         <v>76</v>
       </c>
@@ -3479,10 +3470,10 @@
         <v>15</v>
       </c>
       <c r="E94" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A95" t="s">
         <v>47</v>
       </c>
@@ -3496,10 +3487,10 @@
         <v>15</v>
       </c>
       <c r="E95" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A96" t="s">
         <v>77</v>
       </c>
@@ -3513,15 +3504,15 @@
         <v>15</v>
       </c>
       <c r="E96" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A97" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B97" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C97">
         <v>2</v>
@@ -3530,15 +3521,15 @@
         <v>44</v>
       </c>
       <c r="E97" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A98" t="s">
+        <v>400</v>
+      </c>
+      <c r="B98" t="s">
         <v>402</v>
-      </c>
-      <c r="B98" t="s">
-        <v>404</v>
       </c>
       <c r="C98">
         <v>2</v>
@@ -3547,15 +3538,15 @@
         <v>44</v>
       </c>
       <c r="E98" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A99" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B99" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C99">
         <v>2</v>
@@ -3564,10 +3555,10 @@
         <v>44</v>
       </c>
       <c r="E99" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A100" t="s">
         <v>303</v>
       </c>
@@ -3578,10 +3569,10 @@
         <v>0</v>
       </c>
       <c r="E100" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A101" t="s">
         <v>193</v>
       </c>
@@ -3592,13 +3583,13 @@
         <v>1</v>
       </c>
       <c r="D101" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E101" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A102" t="s">
         <v>194</v>
       </c>
@@ -3609,13 +3600,13 @@
         <v>1</v>
       </c>
       <c r="D102" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E102" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A103" t="s">
         <v>195</v>
       </c>
@@ -3626,13 +3617,13 @@
         <v>1</v>
       </c>
       <c r="D103" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E103" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A104" t="s">
         <v>196</v>
       </c>
@@ -3643,13 +3634,13 @@
         <v>1</v>
       </c>
       <c r="D104" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E104" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A105" t="s">
         <v>197</v>
       </c>
@@ -3660,13 +3651,13 @@
         <v>1</v>
       </c>
       <c r="D105" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E105" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A106" t="s">
         <v>198</v>
       </c>
@@ -3677,13 +3668,13 @@
         <v>1</v>
       </c>
       <c r="D106" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E106" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A107" t="s">
         <v>199</v>
       </c>
@@ -3694,13 +3685,13 @@
         <v>1</v>
       </c>
       <c r="D107" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E107" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A108" t="s">
         <v>200</v>
       </c>
@@ -3711,13 +3702,13 @@
         <v>1</v>
       </c>
       <c r="D108" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E108" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A109" t="s">
         <v>201</v>
       </c>
@@ -3728,13 +3719,13 @@
         <v>1</v>
       </c>
       <c r="D109" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E109" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A110" t="s">
         <v>202</v>
       </c>
@@ -3745,13 +3736,13 @@
         <v>1</v>
       </c>
       <c r="D110" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E110" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A111" t="s">
         <v>203</v>
       </c>
@@ -3762,13 +3753,13 @@
         <v>1</v>
       </c>
       <c r="D111" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E111" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A112" t="s">
         <v>204</v>
       </c>
@@ -3779,13 +3770,13 @@
         <v>1</v>
       </c>
       <c r="D112" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E112" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A113" t="s">
         <v>205</v>
       </c>
@@ -3796,13 +3787,13 @@
         <v>1</v>
       </c>
       <c r="D113" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E113" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A114" t="s">
         <v>206</v>
       </c>
@@ -3813,13 +3804,13 @@
         <v>1</v>
       </c>
       <c r="D114" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E114" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A115" t="s">
         <v>207</v>
       </c>
@@ -3830,13 +3821,13 @@
         <v>1</v>
       </c>
       <c r="D115" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E115" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A116" t="s">
         <v>208</v>
       </c>
@@ -3850,7 +3841,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A117" t="s">
         <v>210</v>
       </c>
@@ -3864,7 +3855,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A118" t="s">
         <v>211</v>
       </c>
@@ -3878,7 +3869,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A119" t="s">
         <v>212</v>
       </c>
@@ -3892,9 +3883,9 @@
         <v>234</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A120" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="B120" t="s">
         <v>209</v>
@@ -3906,7 +3897,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A121" t="s">
         <v>213</v>
       </c>
@@ -3920,7 +3911,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A122" t="s">
         <v>214</v>
       </c>
@@ -3934,7 +3925,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A123" t="s">
         <v>215</v>
       </c>
@@ -3948,7 +3939,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A124" t="s">
         <v>170</v>
       </c>
@@ -3965,7 +3956,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A125" t="s">
         <v>171</v>
       </c>
@@ -3982,7 +3973,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A126" t="s">
         <v>55</v>
       </c>
@@ -3996,7 +3987,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A127" t="s">
         <v>57</v>
       </c>
@@ -4010,7 +4001,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A128" t="s">
         <v>58</v>
       </c>
@@ -4024,7 +4015,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A129" t="s">
         <v>59</v>
       </c>
@@ -4038,7 +4029,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A130" t="s">
         <v>60</v>
       </c>
@@ -4052,7 +4043,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A131" t="s">
         <v>61</v>
       </c>
@@ -4066,7 +4057,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A132" t="s">
         <v>62</v>
       </c>
@@ -4080,7 +4071,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A133" t="s">
         <v>63</v>
       </c>
@@ -4094,7 +4085,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A134" t="s">
         <v>298</v>
       </c>
@@ -4108,7 +4099,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A135" t="s">
         <v>299</v>
       </c>
@@ -4122,7 +4113,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A136" t="s">
         <v>67</v>
       </c>
@@ -4136,7 +4127,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A137" t="s">
         <v>308</v>
       </c>
@@ -4150,7 +4141,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A138" t="s">
         <v>65</v>
       </c>
@@ -4164,7 +4155,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A139" t="s">
         <v>66</v>
       </c>
@@ -4178,7 +4169,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A140" t="s">
         <v>309</v>
       </c>
@@ -4192,7 +4183,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A141" t="s">
         <v>310</v>
       </c>
@@ -4206,7 +4197,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A142" t="s">
         <v>312</v>
       </c>
@@ -4220,7 +4211,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A143" t="s">
         <v>313</v>
       </c>
@@ -4234,7 +4225,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A144" t="s">
         <v>314</v>
       </c>
@@ -4248,7 +4239,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A145" t="s">
         <v>315</v>
       </c>
@@ -4262,7 +4253,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A146" t="s">
         <v>316</v>
       </c>
@@ -4276,7 +4267,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A147" t="s">
         <v>317</v>
       </c>
@@ -4290,7 +4281,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A148" t="s">
         <v>68</v>
       </c>
@@ -4304,7 +4295,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A149" t="s">
         <v>69</v>
       </c>
@@ -4318,7 +4309,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A150" t="s">
         <v>318</v>
       </c>
@@ -4332,7 +4323,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A151" t="s">
         <v>70</v>
       </c>
@@ -4346,7 +4337,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A152" t="s">
         <v>319</v>
       </c>
@@ -4360,7 +4351,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A153" t="s">
         <v>320</v>
       </c>
@@ -4374,7 +4365,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A154" t="s">
         <v>321</v>
       </c>
@@ -4388,7 +4379,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A155" t="s">
         <v>71</v>
       </c>
@@ -4402,7 +4393,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="156" spans="1:5" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" ht="15.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A156" t="s">
         <v>72</v>
       </c>
@@ -4416,7 +4407,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A157" t="s">
         <v>73</v>
       </c>
@@ -4430,7 +4421,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A158" t="s">
         <v>78</v>
       </c>
@@ -4447,9 +4438,9 @@
         <v>237</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A159" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="B159" t="s">
         <v>79</v>
@@ -4464,9 +4455,9 @@
         <v>237</v>
       </c>
     </row>
-    <row r="160" spans="1:5" ht="12.4" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" ht="12.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A160" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="B160" t="s">
         <v>79</v>
@@ -4481,7 +4472,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A161" t="s">
         <v>87</v>
       </c>
@@ -4498,7 +4489,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A162" t="s">
         <v>88</v>
       </c>
@@ -4515,7 +4506,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A163" t="s">
         <v>81</v>
       </c>
@@ -4532,7 +4523,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A164" t="s">
         <v>91</v>
       </c>
@@ -4549,7 +4540,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A165" t="s">
         <v>93</v>
       </c>
@@ -4566,7 +4557,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A166" t="s">
         <v>322</v>
       </c>
@@ -4583,7 +4574,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A167" t="s">
         <v>84</v>
       </c>
@@ -4600,7 +4591,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A168" t="s">
         <v>89</v>
       </c>
@@ -4617,7 +4608,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A169" t="s">
         <v>85</v>
       </c>
@@ -4634,7 +4625,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A170" t="s">
         <v>216</v>
       </c>
@@ -4648,7 +4639,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A171" t="s">
         <v>217</v>
       </c>
@@ -4662,7 +4653,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A172" t="s">
         <v>218</v>
       </c>
@@ -4676,7 +4667,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A173" t="s">
         <v>219</v>
       </c>
@@ -4690,7 +4681,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A174" t="s">
         <v>94</v>
       </c>
@@ -4704,7 +4695,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A175" t="s">
         <v>220</v>
       </c>
@@ -4718,7 +4709,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A176" t="s">
         <v>96</v>
       </c>
@@ -4732,7 +4723,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A177" t="s">
         <v>221</v>
       </c>
@@ -4746,7 +4737,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A178" t="s">
         <v>101</v>
       </c>
@@ -4763,7 +4754,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A179" t="s">
         <v>102</v>
       </c>
@@ -4780,7 +4771,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A180" t="s">
         <v>100</v>
       </c>
@@ -4797,7 +4788,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A181" t="s">
         <v>97</v>
       </c>
@@ -4814,7 +4805,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A182" t="s">
         <v>103</v>
       </c>
@@ -4831,7 +4822,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A183" t="s">
         <v>105</v>
       </c>
@@ -4848,7 +4839,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A184" t="s">
         <v>106</v>
       </c>
@@ -4865,12 +4856,12 @@
         <v>240</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A185" t="s">
         <v>107</v>
       </c>
       <c r="B185" t="s">
-        <v>323</v>
+        <v>443</v>
       </c>
       <c r="C185">
         <v>2</v>
@@ -4879,15 +4870,15 @@
         <v>15</v>
       </c>
       <c r="E185" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A186" t="s">
         <v>114</v>
       </c>
       <c r="B186" t="s">
-        <v>323</v>
+        <v>443</v>
       </c>
       <c r="C186">
         <v>2</v>
@@ -4896,15 +4887,15 @@
         <v>11</v>
       </c>
       <c r="E186" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A187" t="s">
         <v>108</v>
       </c>
       <c r="B187" t="s">
-        <v>324</v>
+        <v>443</v>
       </c>
       <c r="C187">
         <v>2</v>
@@ -4913,15 +4904,15 @@
         <v>15</v>
       </c>
       <c r="E187" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A188" t="s">
         <v>115</v>
       </c>
       <c r="B188" t="s">
-        <v>324</v>
+        <v>443</v>
       </c>
       <c r="C188">
         <v>2</v>
@@ -4930,15 +4921,15 @@
         <v>11</v>
       </c>
       <c r="E188" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A189" t="s">
         <v>109</v>
       </c>
       <c r="B189" t="s">
-        <v>324</v>
+        <v>443</v>
       </c>
       <c r="C189">
         <v>2</v>
@@ -4947,10 +4938,10 @@
         <v>18</v>
       </c>
       <c r="E189" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A190" t="s">
         <v>119</v>
       </c>
@@ -4967,7 +4958,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A191" t="s">
         <v>121</v>
       </c>
@@ -4984,7 +4975,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A192" t="s">
         <v>122</v>
       </c>
@@ -5001,7 +4992,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A193" t="s">
         <v>124</v>
       </c>
@@ -5018,7 +5009,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A194" t="s">
         <v>123</v>
       </c>
@@ -5035,7 +5026,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A195" t="s">
         <v>120</v>
       </c>
@@ -5052,7 +5043,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A196" t="s">
         <v>116</v>
       </c>
@@ -5069,7 +5060,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A197" t="s">
         <v>118</v>
       </c>
@@ -5086,12 +5077,12 @@
         <v>241</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A198" t="s">
         <v>125</v>
       </c>
       <c r="B198" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C198">
         <v>0</v>
@@ -5100,7 +5091,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A199" t="s">
         <v>126</v>
       </c>
@@ -5117,7 +5108,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A200" t="s">
         <v>128</v>
       </c>
@@ -5134,12 +5125,12 @@
         <v>243</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A201" t="s">
         <v>129</v>
       </c>
       <c r="B201" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C201">
         <v>3</v>
@@ -5151,12 +5142,12 @@
         <v>244</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A202" t="s">
         <v>130</v>
       </c>
       <c r="B202" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C202">
         <v>3</v>
@@ -5168,12 +5159,12 @@
         <v>244</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A203" t="s">
         <v>131</v>
       </c>
       <c r="B203" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C203">
         <v>3</v>
@@ -5185,12 +5176,12 @@
         <v>244</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A204" t="s">
         <v>132</v>
       </c>
       <c r="B204" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C204">
         <v>3</v>
@@ -5202,12 +5193,12 @@
         <v>244</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A205" t="s">
         <v>133</v>
       </c>
       <c r="B205" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C205">
         <v>3</v>
@@ -5219,7 +5210,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A206" t="s">
         <v>134</v>
       </c>
@@ -5236,7 +5227,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A207" t="s">
         <v>136</v>
       </c>
@@ -5253,7 +5244,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A208" t="s">
         <v>137</v>
       </c>
@@ -5270,7 +5261,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A209" t="s">
         <v>111</v>
       </c>
@@ -5287,7 +5278,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A210" t="s">
         <v>110</v>
       </c>
@@ -5304,7 +5295,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A211" t="s">
         <v>112</v>
       </c>
@@ -5321,7 +5312,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A212" t="s">
         <v>113</v>
       </c>
@@ -5338,7 +5329,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A213" t="s">
         <v>144</v>
       </c>
@@ -5355,7 +5346,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A214" t="s">
         <v>143</v>
       </c>
@@ -5372,7 +5363,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A215" t="s">
         <v>146</v>
       </c>
@@ -5389,7 +5380,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A216" t="s">
         <v>147</v>
       </c>
@@ -5406,7 +5397,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A217" t="s">
         <v>148</v>
       </c>
@@ -5423,7 +5414,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A218" t="s">
         <v>149</v>
       </c>
@@ -5440,7 +5431,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A219" t="s">
         <v>145</v>
       </c>
@@ -5457,7 +5448,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A220" t="s">
         <v>141</v>
       </c>
@@ -5474,7 +5465,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A221" t="s">
         <v>142</v>
       </c>
@@ -5491,7 +5482,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A222" t="s">
         <v>139</v>
       </c>
@@ -5508,7 +5499,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A223" t="s">
         <v>150</v>
       </c>
@@ -5525,7 +5516,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A224" t="s">
         <v>152</v>
       </c>
@@ -5542,7 +5533,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A225" t="s">
         <v>154</v>
       </c>
@@ -5559,7 +5550,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A226" t="s">
         <v>155</v>
       </c>
@@ -5576,7 +5567,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A227" t="s">
         <v>156</v>
       </c>
@@ -5593,7 +5584,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A228" t="s">
         <v>222</v>
       </c>
@@ -5607,7 +5598,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A229" t="s">
         <v>224</v>
       </c>
@@ -5621,7 +5612,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A230" t="s">
         <v>225</v>
       </c>
@@ -5635,7 +5626,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A231" t="s">
         <v>226</v>
       </c>
@@ -5649,7 +5640,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A232" t="s">
         <v>157</v>
       </c>
@@ -5666,7 +5657,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A233" t="s">
         <v>159</v>
       </c>
@@ -5683,7 +5674,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A234" t="s">
         <v>162</v>
       </c>
@@ -5700,7 +5691,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A235" t="s">
         <v>163</v>
       </c>
@@ -5717,7 +5708,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A236" t="s">
         <v>158</v>
       </c>
@@ -5734,7 +5725,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A237" t="s">
         <v>160</v>
       </c>
@@ -5751,7 +5742,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A238" t="s">
         <v>161</v>
       </c>
@@ -5768,12 +5759,12 @@
         <v>251</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A239" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B239" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C239">
         <v>2</v>
@@ -5782,15 +5773,15 @@
         <v>15</v>
       </c>
       <c r="E239" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A240" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B240" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C240">
         <v>2</v>
@@ -5799,15 +5790,15 @@
         <v>15</v>
       </c>
       <c r="E240" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A241" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B241" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C241">
         <v>2</v>
@@ -5816,15 +5807,15 @@
         <v>15</v>
       </c>
       <c r="E241" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A242" t="s">
         <v>269</v>
       </c>
       <c r="B242" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C242">
         <v>2</v>
@@ -5833,15 +5824,15 @@
         <v>15</v>
       </c>
       <c r="E242" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A243" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B243" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C243">
         <v>2</v>
@@ -5850,15 +5841,15 @@
         <v>15</v>
       </c>
       <c r="E243" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A244" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B244" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C244">
         <v>2</v>
@@ -5867,15 +5858,15 @@
         <v>15</v>
       </c>
       <c r="E244" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A245" t="s">
         <v>270</v>
       </c>
       <c r="B245" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C245">
         <v>2</v>
@@ -5884,15 +5875,15 @@
         <v>15</v>
       </c>
       <c r="E245" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A246" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B246" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C246">
         <v>2</v>
@@ -5901,15 +5892,15 @@
         <v>15</v>
       </c>
       <c r="E246" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A247" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B247" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C247">
         <v>2</v>
@@ -5918,15 +5909,15 @@
         <v>15</v>
       </c>
       <c r="E247" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A248" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B248" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C248">
         <v>2</v>
@@ -5935,15 +5926,15 @@
         <v>15</v>
       </c>
       <c r="E248" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A249" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B249" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C249">
         <v>2</v>
@@ -5952,32 +5943,32 @@
         <v>11</v>
       </c>
       <c r="E249" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A250" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B250" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C250">
         <v>2</v>
       </c>
       <c r="D250" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="E250" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A251" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B251" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C251">
         <v>2</v>
@@ -5986,15 +5977,15 @@
         <v>18</v>
       </c>
       <c r="E251" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A252" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B252" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C252">
         <v>2</v>
@@ -6003,32 +5994,32 @@
         <v>8</v>
       </c>
       <c r="E252" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A253" t="s">
         <v>164</v>
       </c>
       <c r="B253" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C253">
         <v>2</v>
       </c>
       <c r="D253" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E253" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A254" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B254" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C254">
         <v>2</v>
@@ -6037,15 +6028,15 @@
         <v>3</v>
       </c>
       <c r="E254" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A255" t="s">
         <v>271</v>
       </c>
       <c r="B255" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C255">
         <v>2</v>
@@ -6054,15 +6045,15 @@
         <v>15</v>
       </c>
       <c r="E255" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A256" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B256" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C256">
         <v>2</v>
@@ -6071,15 +6062,15 @@
         <v>11</v>
       </c>
       <c r="E256" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A257" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B257" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C257">
         <v>2</v>
@@ -6088,15 +6079,15 @@
         <v>8</v>
       </c>
       <c r="E257" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A258" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B258" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C258">
         <v>2</v>
@@ -6105,15 +6096,15 @@
         <v>3</v>
       </c>
       <c r="E258" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A259" t="s">
         <v>275</v>
       </c>
       <c r="B259" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C259">
         <v>2</v>
@@ -6122,15 +6113,15 @@
         <v>15</v>
       </c>
       <c r="E259" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A260" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B260" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C260">
         <v>2</v>
@@ -6139,15 +6130,15 @@
         <v>15</v>
       </c>
       <c r="E260" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A261" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B261" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C261">
         <v>2</v>
@@ -6156,15 +6147,15 @@
         <v>11</v>
       </c>
       <c r="E261" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A262" t="s">
         <v>167</v>
       </c>
       <c r="B262" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C262">
         <v>2</v>
@@ -6173,32 +6164,32 @@
         <v>8</v>
       </c>
       <c r="E262" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A263" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B263" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C263">
         <v>2</v>
       </c>
       <c r="D263" t="s">
+        <v>380</v>
+      </c>
+      <c r="E263" t="s">
         <v>382</v>
       </c>
-      <c r="E263" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A264" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B264" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C264">
         <v>2</v>
@@ -6207,15 +6198,15 @@
         <v>3</v>
       </c>
       <c r="E264" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A265" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B265" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C265">
         <v>2</v>
@@ -6224,15 +6215,15 @@
         <v>15</v>
       </c>
       <c r="E265" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A266" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B266" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C266">
         <v>2</v>
@@ -6241,15 +6232,15 @@
         <v>11</v>
       </c>
       <c r="E266" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A267" t="s">
         <v>165</v>
       </c>
       <c r="B267" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C267">
         <v>2</v>
@@ -6258,32 +6249,32 @@
         <v>8</v>
       </c>
       <c r="E267" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A268" t="s">
         <v>166</v>
       </c>
       <c r="B268" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C268">
         <v>2</v>
       </c>
       <c r="D268" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E268" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A269" t="s">
         <v>274</v>
       </c>
       <c r="B269" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C269">
         <v>2</v>
@@ -6292,15 +6283,15 @@
         <v>3</v>
       </c>
       <c r="E269" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A270" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B270" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C270">
         <v>2</v>
@@ -6309,15 +6300,15 @@
         <v>8</v>
       </c>
       <c r="E270" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A271" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B271" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C271">
         <v>2</v>
@@ -6326,15 +6317,15 @@
         <v>8</v>
       </c>
       <c r="E271" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="272" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A272" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B272" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C272">
         <v>2</v>
@@ -6343,15 +6334,15 @@
         <v>3</v>
       </c>
       <c r="E272" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A273" t="s">
         <v>276</v>
       </c>
       <c r="B273" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C273">
         <v>2</v>
@@ -6360,15 +6351,15 @@
         <v>15</v>
       </c>
       <c r="E273" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A274" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B274" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C274">
         <v>2</v>
@@ -6377,15 +6368,15 @@
         <v>11</v>
       </c>
       <c r="E274" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="275" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A275" t="s">
         <v>168</v>
       </c>
       <c r="B275" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C275">
         <v>2</v>
@@ -6394,32 +6385,32 @@
         <v>8</v>
       </c>
       <c r="E275" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A276" t="s">
         <v>169</v>
       </c>
       <c r="B276" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C276">
         <v>2</v>
       </c>
       <c r="D276" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E276" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="277" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A277" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B277" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C277">
         <v>2</v>
@@ -6428,15 +6419,15 @@
         <v>3</v>
       </c>
       <c r="E277" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="278" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A278" t="s">
         <v>277</v>
       </c>
       <c r="B278" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C278">
         <v>2</v>
@@ -6445,15 +6436,15 @@
         <v>15</v>
       </c>
       <c r="E278" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="279" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A279" t="s">
         <v>278</v>
       </c>
       <c r="B279" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C279">
         <v>2</v>
@@ -6462,15 +6453,15 @@
         <v>15</v>
       </c>
       <c r="E279" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="280" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A280" t="s">
         <v>279</v>
       </c>
       <c r="B280" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C280">
         <v>2</v>
@@ -6479,15 +6470,15 @@
         <v>15</v>
       </c>
       <c r="E280" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="281" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A281" t="s">
         <v>280</v>
       </c>
       <c r="B281" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C281">
         <v>2</v>
@@ -6496,15 +6487,15 @@
         <v>15</v>
       </c>
       <c r="E281" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="282" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A282" t="s">
         <v>281</v>
       </c>
       <c r="B282" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C282">
         <v>2</v>
@@ -6513,15 +6504,15 @@
         <v>15</v>
       </c>
       <c r="E282" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="283" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A283" t="s">
         <v>265</v>
       </c>
       <c r="B283" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C283">
         <v>2</v>
@@ -6530,15 +6521,15 @@
         <v>15</v>
       </c>
       <c r="E283" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="284" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A284" t="s">
         <v>266</v>
       </c>
       <c r="B284" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C284">
         <v>2</v>
@@ -6547,15 +6538,15 @@
         <v>15</v>
       </c>
       <c r="E284" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="285" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="285" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A285" t="s">
         <v>267</v>
       </c>
       <c r="B285" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C285">
         <v>2</v>
@@ -6564,15 +6555,15 @@
         <v>3</v>
       </c>
       <c r="E285" s="1" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="286" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A286" t="s">
         <v>262</v>
       </c>
       <c r="B286" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C286">
         <v>2</v>
@@ -6581,15 +6572,15 @@
         <v>15</v>
       </c>
       <c r="E286" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="287" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A287" t="s">
         <v>263</v>
       </c>
       <c r="B287" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C287">
         <v>2</v>
@@ -6598,15 +6589,15 @@
         <v>15</v>
       </c>
       <c r="E287" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="288" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A288" t="s">
         <v>264</v>
       </c>
       <c r="B288" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C288">
         <v>2</v>
@@ -6615,15 +6606,15 @@
         <v>15</v>
       </c>
       <c r="E288" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="289" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A289" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B289" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C289">
         <v>2</v>
@@ -6632,15 +6623,15 @@
         <v>15</v>
       </c>
       <c r="E289" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="290" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A290" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B290" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C290">
         <v>2</v>
@@ -6649,15 +6640,15 @@
         <v>11</v>
       </c>
       <c r="E290" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="291" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A291" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B291" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C291">
         <v>2</v>
@@ -6666,15 +6657,15 @@
         <v>8</v>
       </c>
       <c r="E291" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A292" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B292" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C292">
         <v>2</v>
@@ -6683,15 +6674,15 @@
         <v>3</v>
       </c>
       <c r="E292" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A293" t="s">
         <v>311</v>
       </c>
       <c r="B293" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C293">
         <v>2</v>
@@ -6700,15 +6691,15 @@
         <v>15</v>
       </c>
       <c r="E293" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="294" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A294" t="s">
         <v>272</v>
       </c>
       <c r="B294" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C294">
         <v>2</v>
@@ -6717,15 +6708,15 @@
         <v>15</v>
       </c>
       <c r="E294" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="295" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A295" t="s">
         <v>273</v>
       </c>
       <c r="B295" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C295">
         <v>2</v>
@@ -6734,15 +6725,15 @@
         <v>15</v>
       </c>
       <c r="E295" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A296" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B296" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C296">
         <v>2</v>
@@ -6751,15 +6742,15 @@
         <v>15</v>
       </c>
       <c r="E296" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="297" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A297" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B297" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C297">
         <v>1</v>
@@ -6768,15 +6759,15 @@
         <v>15</v>
       </c>
       <c r="E297" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A298" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B298" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C298">
         <v>2</v>
@@ -6785,15 +6776,15 @@
         <v>8</v>
       </c>
       <c r="E298" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="299" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A299" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B299" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C299">
         <v>2</v>
@@ -6802,10 +6793,10 @@
         <v>3</v>
       </c>
       <c r="E299" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="300" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A300" t="s">
         <v>228</v>
       </c>
@@ -6819,7 +6810,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A301" t="s">
         <v>229</v>
       </c>
@@ -6833,7 +6824,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A302" t="s">
         <v>172</v>
       </c>
@@ -6850,7 +6841,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A303" t="s">
         <v>174</v>
       </c>

</xml_diff>